<commit_message>
Update course plans and analyses for ISLL and IKS programs
- Revised quality notes in KAPSG, KFPPG, KLJMG, KMLJG, KMMPG, KMPTG, and KMUSG course plans to reflect updated course references and corrections.
- Added detailed notes on discontinued courses in various program analyses.
- Updated binary files for course-related documents including Excel sheets for course planning and analysis.
- Corrected language and formatting issues in course descriptions for clarity and consistency.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/03 IKS/Analys/Nedlagda kursreferenser.xlsx
+++ b/vault-dalarna-university/03 IKS/Analys/Nedlagda kursreferenser.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Nedlagda kursreferenser" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Nedlagda kursreferenser'!$A$1:$G$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Nedlagda kursreferenser'!$A$1:$G$33</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>KFTPG</t>
+          <t>KAPSG</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -494,14 +494,10 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2014-03-19</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2021-03-23</t>
-        </is>
-      </c>
+          <t>2023-01-30</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>Programmet listar nedlagd kurs</t>
@@ -509,19 +505,19 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>`Konceptutveckling inom medieproduktion` → `BQ2049` (nedlagd 2025-03-06) — plain-text-referens</t>
+          <t>`Introduktion till audiovisuell produktion` → `GLP239` (nedlagd 2026-06-25) — wikilink-länk till nedlagd kod</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KFTPG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KAPSG</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>LBF3A</t>
+          <t>KAPSG</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -531,14 +527,10 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2020-12-17</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2023-06-02</t>
-        </is>
-      </c>
+          <t>2023-01-30</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>Programmet listar nedlagd kurs</t>
@@ -546,19 +538,19 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>`Text, kommunikation och lärande i en mångkulturell skola` → `GSV22L` (nedlagd 2024-10-11) — plain-text-referens</t>
+          <t>`Audiovisuellt berättande` → `GLP23B` (nedlagd 2026-06-25) — wikilink-länk till nedlagd kod</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LBF3A</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KAPSG</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>LP79A</t>
+          <t>KAPSG</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -568,14 +560,10 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2017-12-19</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2022-08-29</t>
-        </is>
-      </c>
+          <t>2023-01-30</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>Programmet listar nedlagd kurs</t>
@@ -583,19 +571,19 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>`Didaktik och ledarskap för ämneslärare` → `PG1020` (nedlagd 2018-07-02) — plain-text-referens</t>
+          <t>`Audiovisuell komposition` → `GLP23A` (nedlagd 2026-06-25) — wikilink-länk till nedlagd kod</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LP79A</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KAPSG</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>LPGYA</t>
+          <t>KAPSG</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -605,14 +593,10 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2017-12-19</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2022-08-29</t>
-        </is>
-      </c>
+          <t>2023-01-30</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>Programmet listar nedlagd kurs</t>
@@ -620,19 +604,19 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>`Didaktik och ledarskap för ämneslärare` → `PG1020` (nedlagd 2018-07-02) — plain-text-referens</t>
+          <t>`Audiovisuell gestaltning` → `GLP234` (nedlagd 2026-06-25) — wikilink-länk till nedlagd kod</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LPGYA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KAPSG</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>SSHVG</t>
+          <t>KAPSG</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -642,7 +626,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2021-06-16</t>
+          <t>2023-01-30</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -653,19 +637,19 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>`Samhällsekonomi` → `GSQ25R` (nedlagd 2025-12-08) — plain-text-referens</t>
+          <t>`Vetenskaplig uppsats i Ljud- och musikproduktion` → `LP1065` (nedlagd 2026-06-25) — wikilink-länk till nedlagd kod</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KAPSG</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>SSHVG</t>
+          <t>KAPSG</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -675,7 +659,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2021-06-16</t>
+          <t>2023-01-30</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -686,19 +670,19 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>`Konformitet och avvikelse` → `SO1007` (nedlagd 2025-11-13) — plain-text-referens</t>
+          <t>`Audiovisuella installationer` → `GLP235` (nedlagd 2026-06-25) — wikilink-länk till nedlagd kod</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KAPSG</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>STMGG</t>
+          <t>KAPSG</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -708,14 +692,10 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2017-11-15</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>2023-03-17</t>
-        </is>
-      </c>
+          <t>2023-01-30</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>Programmet listar nedlagd kurs</t>
@@ -723,19 +703,19 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>`Grundläggande ekonomistyrning` → `FEA034` (nedlagd 2008-03-18) — plain-text-referens</t>
+          <t>`Audiovisuell performance` → `GLP236` (nedlagd 2026-06-25) — wikilink-länk till nedlagd kod</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=STMGG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KAPSG</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>STMGG</t>
+          <t>KAPSG</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -745,14 +725,10 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2017-11-15</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>2023-03-17</t>
-        </is>
-      </c>
+          <t>2023-01-30</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>Programmet listar nedlagd kurs</t>
@@ -760,54 +736,877 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>`Kvalitativa forskningsmetoder` → `SB3002` (nedlagd 2013-01-15) — plain-text-referens</t>
+          <t>`Kommunikationsteorier` → `GLP2MS` (nedlagd 2026-06-25) — wikilink-länk till nedlagd kod</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=STMGG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KAPSG</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>KAPSG</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2023-01-30</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Programmet listar nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>`Arbetsplatsförlagd utbildning i medieproduktion` → `GLP2QD` (nedlagd 2026-06-25) — wikilink-länk till nedlagd kod</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KAPSG</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>KFPPG</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2025-01-15</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Programmet listar nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>`Introduktion till medieproduktion` → `GLP2FH` (nedlagd 2026-06-25) — wikilink-länk till nedlagd kod</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KFPPG</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>KFTPG</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2014-03-19</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2021-03-23</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Programmet listar nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>`Konceptutveckling inom medieproduktion` → `BQ2049` (nedlagd 2025-03-06) — plain-text-referens</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KFTPG</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>KLJMG</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2021-03-23</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2023-07-05</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Programmet listar nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>`Introduktion till medieproduktion` → `GLP2FH` (nedlagd 2026-06-25) — wikilink-länk till nedlagd kod</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KLJMG</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>KLJMG</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2021-03-23</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2023-07-05</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Programmet listar nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>`Audioteknologi 1` → `GLP29R` (nedlagd 2026-06-25) — wikilink-länk till nedlagd kod</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KLJMG</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>KLJMG</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2021-03-23</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2023-07-05</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Programmet listar nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>`Ljudteori` → `GLP2FP` (nedlagd 2026-06-25) — wikilink-länk till nedlagd kod</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KLJMG</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>KLJMG</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2021-03-23</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2023-07-05</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Programmet listar nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>`Ljudskapande till rörliga bilder` → `GLP29S` (nedlagd 2026-06-25) — wikilink-länk till nedlagd kod</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KLJMG</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>KLJMG</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2021-03-23</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2023-07-05</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Programmet listar nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>`Inspelning i studio` → `GLP2QU` (nedlagd 2026-06-25) — wikilink-länk till nedlagd kod</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KLJMG</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>KLJMG</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2021-03-23</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2023-07-05</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Programmet listar nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>`Audioteknologi 2` → `LP1080` (nedlagd 2026-06-25) — wikilink-länk till nedlagd kod</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KLJMG</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>KLJMG</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2021-03-23</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2023-07-05</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Programmet listar nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>`Vetenskaplig uppsats i Ljud- och musikproduktion` → `LP1065` (nedlagd 2026-06-25) — wikilink-länk till nedlagd kod</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KLJMG</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>KLJMG</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2021-03-23</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2023-07-05</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Programmet listar nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>`Produktionsprocesser och -villkor inom musikproduktion` → `LP1072` (nedlagd 2026-06-25) — wikilink-länk till nedlagd kod</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KLJMG</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>KMLJG</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2020-10-20</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2023-07-05</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Programmet listar nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>`Ljudteori` → `GLP2FP` (nedlagd 2026-06-25) — wikilink-länk till nedlagd kod</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KMLJG</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>KMLJG</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2020-10-20</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>2023-07-05</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Programmet listar nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>`Inspelning i studio` → `GLP2QU` (nedlagd 2026-06-25) — wikilink-länk till nedlagd kod</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KMLJG</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>KMMPG</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2025-01-15</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Programmet listar nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>`Introduktion till medieproduktion` → `GLP2FH` (nedlagd 2026-06-25) — wikilink-länk till nedlagd kod</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KMMPG</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>KMPTG</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2025-01-15</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Programmet listar nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>`Introduktion till medieproduktion` → `GLP2FH` (nedlagd 2026-06-25) — wikilink-länk till nedlagd kod</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KMPTG</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>KMUSG</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2025-01-15</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Programmet listar nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>`Introduktion till medieproduktion` → `GLP2FH` (nedlagd 2026-06-25) — wikilink-länk till nedlagd kod</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KMUSG</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>LBF3A</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2020-12-17</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>2023-06-02</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Programmet listar nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>`Text, kommunikation och lärande i en mångkulturell skola` → `GSV22L` (nedlagd 2024-10-11) — plain-text-referens</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LBF3A</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>LP79A</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2017-12-19</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>2022-08-29</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Programmet listar nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>`Didaktik och ledarskap för ämneslärare` → `PG1020` (nedlagd 2018-07-02) — plain-text-referens</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LP79A</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>LPGYA</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2017-12-19</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>2022-08-29</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Programmet listar nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>`Didaktik och ledarskap för ämneslärare` → `PG1020` (nedlagd 2018-07-02) — plain-text-referens</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LPGYA</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>SSHVG</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>2021-06-16</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Programmet listar nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>`Samhällsekonomi` → `GSQ25R` (nedlagd 2025-12-08) — plain-text-referens</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>SSHVG</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>2021-06-16</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Programmet listar nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>`Konformitet och avvikelse` → `SO1007` (nedlagd 2025-11-13) — plain-text-referens</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
           <t>STMGG</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
         <is>
           <t>2017-11-15</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>2023-03-17</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Programmet listar nedlagd kurs</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Programmet listar nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>`Grundläggande ekonomistyrning` → `FEA034` (nedlagd 2008-03-18) — plain-text-referens</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=STMGG</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>STMGG</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>2017-11-15</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>2023-03-17</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Programmet listar nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>`Kvalitativa forskningsmetoder` → `SB3002` (nedlagd 2013-01-15) — plain-text-referens</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=STMGG</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>STMGG</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>2017-11-15</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>2023-03-17</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Programmet listar nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
         <is>
           <t>`Projektarbete` → `BTA009` (nedlagd 2008-05-22) — plain-text-referens</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=STMGG</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G10"/>
+  <autoFilter ref="A1:G33"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
@@ -827,6 +1626,52 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A20" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A21" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A23" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A24" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A25" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A26" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A27" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A28" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A29" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A30" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A31" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A33" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId64"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>